<commit_message>
fix(tests): resolve method name mismatch in explore spec; achieve 100% test pass rate across all suites
</commit_message>
<xml_diff>
--- a/selenium-tests/reports/selenium_e2e_test_report.xlsx
+++ b/selenium-tests/reports/selenium_e2e_test_report.xlsx
@@ -35,7 +35,7 @@
     <t>Execution Date</t>
   </si>
   <si>
-    <t>22/7/2026, 5:36:17 pm</t>
+    <t>22/7/2026, 6:44:00 pm</t>
   </si>
   <si>
     <t>Browser / Mode</t>
@@ -47,7 +47,7 @@
     <t>Total Duration</t>
   </si>
   <si>
-    <t>0.02 seconds</t>
+    <t>0.03 seconds</t>
   </si>
   <si>
     <t>Selenium Test Execution Summary Metrics</t>
@@ -98,7 +98,7 @@
     <t>PASS</t>
   </si>
   <si>
-    <t>5:36:17 pm</t>
+    <t>6:44:00 pm</t>
   </si>
   <si>
     <t>N/A</t>
@@ -864,7 +864,7 @@
         <v>27</v>
       </c>
       <c r="E4" s="11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F4" s="9" t="s">
         <v>28</v>

</xml_diff>